<commit_message>
temp: full audit report
</commit_message>
<xml_diff>
--- a/audit_full_system.xlsx
+++ b/audit_full_system.xlsx
@@ -515,7 +515,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
@@ -555,7 +555,7 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
@@ -575,7 +575,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
@@ -774,11 +774,11 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>77736</v>
+        <v>79030</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>234</t>
+          <t>2345</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -797,13 +797,13 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>234</v>
+        <v>23</v>
       </c>
       <c r="G2" t="n">
-        <v>234</v>
+        <v>23</v>
       </c>
       <c r="H2" t="n">
-        <v>234</v>
+        <v>23</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -823,11 +823,11 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>94391</v>
+        <v>94396</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>1223</t>
+          <t>123</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -856,7 +856,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Bybit</t>
+          <t>MEXC</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -872,11 +872,11 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>94396</v>
+        <v>77736</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>123</t>
+          <t>234</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -891,21 +891,21 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>TON</t>
+          <t>USDT</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>123</v>
+        <v>234</v>
       </c>
       <c r="G4" t="n">
-        <v>123</v>
+        <v>234</v>
       </c>
       <c r="H4" t="n">
-        <v>123</v>
+        <v>234</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>MEXC</t>
+          <t>Bybit</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -921,11 +921,11 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>79030</v>
+        <v>94391</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2345</t>
+          <t>1223</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -940,17 +940,17 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>USDT</t>
+          <t>TON</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>23</v>
+        <v>123</v>
       </c>
       <c r="G5" t="n">
-        <v>23</v>
+        <v>123</v>
       </c>
       <c r="H5" t="n">
-        <v>23</v>
+        <v>123</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -2768,7 +2768,7 @@
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>50073</v>
+        <v>50074</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2817,7 +2817,7 @@
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>50074</v>
+        <v>50073</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -3062,7 +3062,7 @@
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>63505</v>
+        <v>63504</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3111,7 +3111,7 @@
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>63504</v>
+        <v>63505</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3209,7 +3209,7 @@
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>52408</v>
+        <v>52387</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -3258,7 +3258,7 @@
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>52387</v>
+        <v>52408</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3405,7 +3405,7 @@
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>63585</v>
+        <v>63587</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
@@ -3454,7 +3454,7 @@
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>63587</v>
+        <v>63585</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
@@ -3503,11 +3503,11 @@
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>69018</v>
+        <v>63771</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>OB-1D8XQAAK4L</t>
+          <t>OB-MYN32CNAL0</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -3526,13 +3526,13 @@
         </is>
       </c>
       <c r="F49" t="n">
-        <v>198.2161</v>
+        <v>121.3815</v>
       </c>
       <c r="G49" t="n">
-        <v>80.31999999999999</v>
+        <v>81.65000000000001</v>
       </c>
       <c r="H49" t="n">
-        <v>16064</v>
+        <v>10000</v>
       </c>
       <c r="I49" t="inlineStr">
         <is>
@@ -3546,17 +3546,17 @@
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>Дубль: 2 ордеров с одинаковым ID биржи 'OB-1D8XQAAK4L'</t>
+          <t>Дубль: 2 ордеров с одинаковым ID биржи 'OB-MYN32CNAL0'</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>69017</v>
+        <v>63759</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>OB-1D8XQAAK4L</t>
+          <t>OB-MYN32CNAL0</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -3575,13 +3575,13 @@
         </is>
       </c>
       <c r="F50" t="n">
-        <v>198.2161</v>
+        <v>142.7156</v>
       </c>
       <c r="G50" t="n">
-        <v>80.31999999999999</v>
+        <v>81.65000000000001</v>
       </c>
       <c r="H50" t="n">
-        <v>16064</v>
+        <v>11758</v>
       </c>
       <c r="I50" t="inlineStr">
         <is>
@@ -3590,12 +3590,12 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>27.03.2026 16:02</t>
+          <t>20.03.2026 14:02</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>Дубль: 2 ордеров с одинаковым ID биржи 'OB-1D8XQAAK4L'</t>
+          <t>Дубль: 2 ордеров с одинаковым ID биржи 'OB-MYN32CNAL0'</t>
         </is>
       </c>
     </row>
@@ -3699,11 +3699,11 @@
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>63771</v>
+        <v>69018</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>OB-MYN32CNAL0</t>
+          <t>OB-1D8XQAAK4L</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -3722,13 +3722,13 @@
         </is>
       </c>
       <c r="F53" t="n">
-        <v>121.3815</v>
+        <v>198.2161</v>
       </c>
       <c r="G53" t="n">
-        <v>81.65000000000001</v>
+        <v>80.31999999999999</v>
       </c>
       <c r="H53" t="n">
-        <v>10000</v>
+        <v>16064</v>
       </c>
       <c r="I53" t="inlineStr">
         <is>
@@ -3742,17 +3742,17 @@
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>Дубль: 2 ордеров с одинаковым ID биржи 'OB-MYN32CNAL0'</t>
+          <t>Дубль: 2 ордеров с одинаковым ID биржи 'OB-1D8XQAAK4L'</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>63759</v>
+        <v>69017</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>OB-MYN32CNAL0</t>
+          <t>OB-1D8XQAAK4L</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -3771,13 +3771,13 @@
         </is>
       </c>
       <c r="F54" t="n">
-        <v>142.7156</v>
+        <v>198.2161</v>
       </c>
       <c r="G54" t="n">
-        <v>81.65000000000001</v>
+        <v>80.31999999999999</v>
       </c>
       <c r="H54" t="n">
-        <v>11758</v>
+        <v>16064</v>
       </c>
       <c r="I54" t="inlineStr">
         <is>
@@ -3786,12 +3786,12 @@
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>20.03.2026 14:02</t>
+          <t>27.03.2026 16:02</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>Дубль: 2 ордеров с одинаковым ID биржи 'OB-MYN32CNAL0'</t>
+          <t>Дубль: 2 ордеров с одинаковым ID биржи 'OB-1D8XQAAK4L'</t>
         </is>
       </c>
     </row>
@@ -3895,7 +3895,7 @@
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>63967</v>
+        <v>63968</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
@@ -3944,7 +3944,7 @@
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>63968</v>
+        <v>63967</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
@@ -3993,7 +3993,7 @@
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>64321</v>
+        <v>64320</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
@@ -4042,7 +4042,7 @@
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>64320</v>
+        <v>64321</v>
       </c>
       <c r="B60" t="inlineStr">
         <is>
@@ -4189,7 +4189,7 @@
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>66001</v>
+        <v>66002</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
@@ -4238,7 +4238,7 @@
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>66002</v>
+        <v>66001</v>
       </c>
       <c r="B64" t="inlineStr">
         <is>
@@ -4385,7 +4385,7 @@
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>72314</v>
+        <v>72315</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
@@ -4434,7 +4434,7 @@
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>72315</v>
+        <v>72314</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
@@ -4786,7 +4786,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K23"/>
+  <dimension ref="A1:K20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4959,11 +4959,11 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>77736</v>
+        <v>79030</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>234</t>
+          <t>2345</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -4982,13 +4982,13 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>234</v>
+        <v>23</v>
       </c>
       <c r="G4" t="n">
-        <v>234</v>
+        <v>23</v>
       </c>
       <c r="H4" t="n">
-        <v>234</v>
+        <v>23</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -5002,17 +5002,17 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Курс 234.00 отличается от курса дня на этой же бирже (84.00) на 179%</t>
+          <t>Курс 23.00 отличается от курса дня на этой же бирже (84.00) на 73%</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>79030</v>
+        <v>77736</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2345</t>
+          <t>234</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -5031,13 +5031,13 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>23</v>
+        <v>234</v>
       </c>
       <c r="G5" t="n">
-        <v>23</v>
+        <v>234</v>
       </c>
       <c r="H5" t="n">
-        <v>23</v>
+        <v>234</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -5051,7 +5051,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Курс 23.00 отличается от курса дня на этой же бирже (84.00) на 73%</t>
+          <t>Курс 234.00 отличается от курса дня на этой же бирже (84.00) на 179%</t>
         </is>
       </c>
     </row>
@@ -5204,16 +5204,16 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>114472</v>
+        <v>118516</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>OB-OMKY545FDH</t>
+          <t>OS-JC0TUYBAXY</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>rimkus</t>
+          <t>dron</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -5227,13 +5227,13 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>137.7411</v>
+        <v>238.5781</v>
       </c>
       <c r="G9" t="n">
-        <v>10500</v>
+        <v>8383</v>
       </c>
       <c r="H9" t="n">
-        <v>10500</v>
+        <v>20000</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -5242,32 +5242,32 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>30.04.2026 09:46</t>
+          <t>01.05.2026 14:11</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Курс 10500.00 отличается от курса дня на этой же бирже (83.29) на 12507%</t>
+          <t>Курс 8383.00 отличается от курса дня на этой же бирже (75.40) на 11018%</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>118516</v>
+        <v>125227</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>OS-JC0TUYBAXY</t>
+          <t>OS-G0CNZNGY3M</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>dron</t>
+          <t>salatgereev_adam</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -5276,13 +5276,13 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>238.5781</v>
+        <v>18.1818</v>
       </c>
       <c r="G10" t="n">
-        <v>8383</v>
+        <v>220</v>
       </c>
       <c r="H10" t="n">
-        <v>20000</v>
+        <v>4000</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -5291,32 +5291,32 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>01.05.2026 14:11</t>
+          <t>07.05.2026 22:28</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Курс 8383.00 отличается от курса дня на этой же бирже (75.40) на 11018%</t>
+          <t>Курс 220.00 отличается от курса дня на этой же бирже (82.80) на 166%</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>125227</v>
+        <v>131626</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>OS-G0CNZNGY3M</t>
+          <t>74,36</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>salatgereev_adam</t>
+          <t>rimkus</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -5325,13 +5325,13 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>18.1818</v>
+        <v>187.9267</v>
       </c>
       <c r="G11" t="n">
-        <v>220</v>
+        <v>187.93</v>
       </c>
       <c r="H11" t="n">
-        <v>4000</v>
+        <v>14100</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -5340,32 +5340,32 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>07.05.2026 22:28</t>
+          <t>14.05.2026 10:10</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Курс 220.00 отличается от курса дня на этой же бирже (82.80) на 166%</t>
+          <t>Курс 187.93 отличается от курса дня на этой же бирже (81.40) на 131%</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>131626</v>
+        <v>147203</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>74,36</t>
+          <t>OS-5HSWHDDXZU</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>rimkus</t>
+          <t>kurbatov</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -5374,13 +5374,13 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>187.9267</v>
+        <v>41.96</v>
       </c>
       <c r="G12" t="n">
-        <v>187.93</v>
+        <v>3500</v>
       </c>
       <c r="H12" t="n">
-        <v>14100</v>
+        <v>3500</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -5389,27 +5389,27 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>14.05.2026 10:10</t>
+          <t>14.05.2026 23:53</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Курс 187.93 отличается от курса дня на этой же бирже (81.40) на 131%</t>
+          <t>Курс 3500.00 отличается от курса дня на этой же бирже (81.40) на 4200%</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>147203</v>
+        <v>133219</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>OS-5HSWHDDXZU</t>
+          <t>OS-6P2Y7H5LR7</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>kurbatov</t>
+          <t>arslangereev</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -5423,13 +5423,13 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>41.96</v>
+        <v>83</v>
       </c>
       <c r="G13" t="n">
-        <v>3500</v>
+        <v>313.25</v>
       </c>
       <c r="H13" t="n">
-        <v>3500</v>
+        <v>26000</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -5438,27 +5438,27 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>14.05.2026 23:53</t>
+          <t>15.05.2026 17:40</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Курс 3500.00 отличается от курса дня на этой же бирже (81.40) на 4200%</t>
+          <t>Курс 313.25 отличается от курса дня на этой же бирже (81.39) на 285%</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>133219</v>
+        <v>149614</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>OS-6P2Y7H5LR7</t>
+          <t>OS-5HXMZNG4V2</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>arslangereev</t>
+          <t>kolosov</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -5472,13 +5472,13 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>83</v>
+        <v>24.09</v>
       </c>
       <c r="G14" t="n">
-        <v>313.25</v>
+        <v>24.09</v>
       </c>
       <c r="H14" t="n">
-        <v>26000</v>
+        <v>2000</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -5487,27 +5487,27 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>15.05.2026 17:40</t>
+          <t>27.05.2026 12:48</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Курс 313.25 отличается от курса дня на этой же бирже (81.39) на 285%</t>
+          <t>Курс 24.09 отличается от курса дня на этой же бирже (80.42) на 70%</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>149614</v>
+        <v>165636</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>OS-5HXMZNG4V2</t>
+          <t>d1746241979238882304</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>kolosov</t>
+          <t>vishnyakov_denis</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -5521,37 +5521,37 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>24.09</v>
+        <v>7.5</v>
       </c>
       <c r="G15" t="n">
-        <v>24.09</v>
+        <v>600</v>
       </c>
       <c r="H15" t="n">
-        <v>2000</v>
+        <v>600</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Telegram</t>
+          <t>MEXC</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>27.05.2026 12:48</t>
+          <t>10.06.2026 16:15</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Курс 24.09 отличается от курса дня на этой же бирже (80.42) на 70%</t>
+          <t>Курс 600.00 отличается от курса дня на этой же бирже (79.49) на 655%</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>165636</v>
+        <v>166232</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>d1746241979238882304</t>
+          <t>d1746426851811171328</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -5570,13 +5570,13 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>7.5</v>
+        <v>8.75</v>
       </c>
       <c r="G16" t="n">
-        <v>600</v>
+        <v>700</v>
       </c>
       <c r="H16" t="n">
-        <v>600</v>
+        <v>700</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -5585,32 +5585,32 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>10.06.2026 16:15</t>
+          <t>10.06.2026 22:14</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Курс 600.00 отличается от курса дня на этой же бирже (79.49) на 655%</t>
+          <t>Курс 700.00 отличается от курса дня на этой же бирже (79.49) на 781%</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>166232</v>
+        <v>188170</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>d1746426851811171328</t>
+          <t>OB-TPPY013IP2</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>vishnyakov_denis</t>
+          <t>charaburaev</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -5619,47 +5619,47 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>8.75</v>
+        <v>178.74</v>
       </c>
       <c r="G17" t="n">
-        <v>700</v>
+        <v>13600</v>
       </c>
       <c r="H17" t="n">
-        <v>700</v>
+        <v>13600</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>MEXC</t>
+          <t>Telegram</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>10.06.2026 22:14</t>
+          <t>25.06.2026 14:19</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Курс 700.00 отличается от курса дня на этой же бирже (79.49) на 781%</t>
+          <t>Курс 13600.00 отличается от курса дня на этой же бирже (85.50) на 15806%</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>188170</v>
+        <v>197129</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>OB-TPPY013IP2</t>
+          <t>OS-5TB5J6OEIJ</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>charaburaev</t>
+          <t>dron</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -5668,13 +5668,13 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>178.74</v>
+        <v>30</v>
       </c>
       <c r="G18" t="n">
-        <v>13600</v>
+        <v>152.64</v>
       </c>
       <c r="H18" t="n">
-        <v>13600</v>
+        <v>4579</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -5683,27 +5683,27 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>25.06.2026 14:19</t>
+          <t>02.07.2026 16:33</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Курс 13600.00 отличается от курса дня на этой же бирже (85.50) на 15806%</t>
+          <t>Курс 152.64 отличается от курса дня на этой же бирже (85.20) на 79%</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>192273</v>
+        <v>207432</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>OB-GHT30FAHX1</t>
+          <t>OB-GHWP1CV4QO</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>khabibullin</t>
+          <t>nasibov</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -5717,13 +5717,13 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>128.8998</v>
+        <v>77.66</v>
       </c>
       <c r="G19" t="n">
-        <v>7815</v>
+        <v>140.37</v>
       </c>
       <c r="H19" t="n">
-        <v>10164.18</v>
+        <v>11000</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -5732,27 +5732,27 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>29.06.2026 14:10</t>
+          <t>09.07.2026 11:47</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>Курс 7815.00 отличается от курса дня на этой же бирже (78.44) на 9864%</t>
+          <t>Курс 140.37 отличается от курса дня на этой же бирже (78.60) на 79%</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>197129</v>
+        <v>220732</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>OS-5TB5J6OEIJ</t>
+          <t>OS-FMNLK7Z3ZE</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>dron</t>
+          <t>rodionov</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -5766,13 +5766,13 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>30</v>
+        <v>33.3593</v>
       </c>
       <c r="G20" t="n">
-        <v>152.64</v>
+        <v>23.41</v>
       </c>
       <c r="H20" t="n">
-        <v>4579</v>
+        <v>3000</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -5781,159 +5781,12 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>02.07.2026 16:33</t>
+          <t>18.07.2026 23:41</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Курс 152.64 отличается от курса дня на этой же бирже (85.20) на 79%</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="n">
-        <v>207432</v>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>OB-GHWP1CV4QO</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>nasibov</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>USDT</t>
-        </is>
-      </c>
-      <c r="F21" t="n">
-        <v>77.66</v>
-      </c>
-      <c r="G21" t="n">
-        <v>140.37</v>
-      </c>
-      <c r="H21" t="n">
-        <v>11000</v>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>Telegram</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>09.07.2026 11:47</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>Курс 140.37 отличается от курса дня на этой же бирже (78.60) на 79%</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="n">
-        <v>220732</v>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>OS-FMNLK7Z3ZE</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>rodionov</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>USDT</t>
-        </is>
-      </c>
-      <c r="F22" t="n">
-        <v>33.3593</v>
-      </c>
-      <c r="G22" t="n">
-        <v>23.41</v>
-      </c>
-      <c r="H22" t="n">
-        <v>3000</v>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>Telegram</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>18.07.2026 23:41</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
           <t>Курс 23.41 отличается от курса дня на этой же бирже (88.85) на 74%</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="n">
-        <v>221773</v>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>OS-3KWU45AWNW</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>akhmedov</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>USDT</t>
-        </is>
-      </c>
-      <c r="F23" t="n">
-        <v>10.7527</v>
-      </c>
-      <c r="G23" t="n">
-        <v>1000</v>
-      </c>
-      <c r="H23" t="n">
-        <v>1000</v>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>Telegram</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>19.07.2026 23:38</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>Курс 1000.00 отличается от курса дня на этой же бирже (86.99) на 1050%</t>
         </is>
       </c>
     </row>
@@ -6605,7 +6458,7 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Кол-во в 10 раз больше типичной сделки этого юзера (950.05, без учёта этого ордера)</t>
+          <t>Кол-во в 10 раз больше типичной сделки этого юзера (949.08, без учёта этого ордера)</t>
         </is>
       </c>
     </row>
@@ -6801,7 +6654,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Кол-во в 13 раз больше типичной сделки этого юзера (950.05, без учёта этого ордера)</t>
+          <t>Кол-во в 13 раз больше типичной сделки этого юзера (949.08, без учёта этого ордера)</t>
         </is>
       </c>
     </row>
@@ -7291,7 +7144,7 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>Кол-во в 14 раз больше типичной сделки этого юзера (950.05, без учёта этого ордера)</t>
+          <t>Кол-во в 14 раз больше типичной сделки этого юзера (949.08, без учёта этого ордера)</t>
         </is>
       </c>
     </row>
@@ -7585,7 +7438,7 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>Кол-во в 14 раз больше типичной сделки этого юзера (950.05, без учёта этого ордера)</t>
+          <t>Кол-во в 14 раз больше типичной сделки этого юзера (949.08, без учёта этого ордера)</t>
         </is>
       </c>
     </row>
@@ -7830,7 +7683,7 @@
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>Кол-во в 15 раз больше типичной сделки этого юзера (950.05, без учёта этого ордера)</t>
+          <t>Кол-во в 15 раз больше типичной сделки этого юзера (949.08, без учёта этого ордера)</t>
         </is>
       </c>
     </row>
@@ -8026,7 +7879,7 @@
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>Кол-во в 15 раз больше типичной сделки этого юзера (950.05, без учёта этого ордера)</t>
+          <t>Кол-во в 15 раз больше типичной сделки этого юзера (949.08, без учёта этого ордера)</t>
         </is>
       </c>
     </row>
@@ -8124,7 +7977,7 @@
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>Кол-во в 11 раз больше типичной сделки этого юзера (630.00, без учёта этого ордера)</t>
+          <t>Кол-во в 11 раз больше типичной сделки этого юзера (628.93, без учёта этого ордера)</t>
         </is>
       </c>
     </row>
@@ -8173,7 +8026,7 @@
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>Кол-во в 15 раз больше типичной сделки этого юзера (950.05, без учёта этого ордера)</t>
+          <t>Кол-во в 15 раз больше типичной сделки этого юзера (949.08, без учёта этого ордера)</t>
         </is>
       </c>
     </row>
@@ -8222,7 +8075,7 @@
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>Кол-во в 16 раз больше типичной сделки этого юзера (617.44, без учёта этого ордера)</t>
+          <t>Кол-во в 16 раз больше типичной сделки этого юзера (621.12, без учёта этого ордера)</t>
         </is>
       </c>
     </row>
@@ -8369,7 +8222,7 @@
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>Кол-во в 12 раз больше типичной сделки этого юзера (243.90, без учёта этого ордера)</t>
+          <t>Кол-во в 12 раз больше типичной сделки этого юзера (246.39, без учёта этого ордера)</t>
         </is>
       </c>
     </row>
@@ -8516,7 +8369,7 @@
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>Кол-во в 11 раз больше типичной сделки этого юзера (617.44, без учёта этого ордера)</t>
+          <t>Кол-во в 11 раз больше типичной сделки этого юзера (621.12, без учёта этого ордера)</t>
         </is>
       </c>
     </row>
@@ -8663,7 +8516,7 @@
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>Кол-во в 12 раз больше типичной сделки этого юзера (243.90, без учёта этого ордера)</t>
+          <t>Кол-во в 12 раз больше типичной сделки этого юзера (246.39, без учёта этого ордера)</t>
         </is>
       </c>
     </row>
@@ -9202,7 +9055,7 @@
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>Кол-во в 11 раз больше типичной сделки этого юзера (461.89, без учёта этого ордера)</t>
+          <t>Кол-во в 11 раз больше типичной сделки этого юзера (467.15, без учёта этого ордера)</t>
         </is>
       </c>
     </row>
@@ -9545,7 +9398,7 @@
       </c>
       <c r="K73" t="inlineStr">
         <is>
-          <t>Кол-во в 12 раз больше типичной сделки этого юзера (150.00, без учёта этого ордера)</t>
+          <t>Кол-во в 12 раз больше типичной сделки этого юзера (150.66, без учёта этого ордера)</t>
         </is>
       </c>
     </row>
@@ -9707,7 +9560,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9782,21 +9635,21 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>114472</v>
+        <v>147203</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>OB-OMKY545FDH</t>
+          <t>OS-5HSWHDDXZU</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>rimkus</t>
+          <t>kurbatov</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -9805,13 +9658,13 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>137.7411</v>
+        <v>41.96</v>
       </c>
       <c r="G2" t="n">
-        <v>10500</v>
+        <v>3500</v>
       </c>
       <c r="H2" t="n">
-        <v>10500</v>
+        <v>3500</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -9820,32 +9673,32 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>30.04.2026 09:46</t>
+          <t>14.05.2026 23:53</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Похоже, в поле 'Курс' вписана сумма сделки (10500.00) вместо реального курса</t>
+          <t>Похоже, в поле 'Курс' вписана сумма сделки (3500.00) вместо реального курса</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>147203</v>
+        <v>188170</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>OS-5HSWHDDXZU</t>
+          <t>OB-TPPY013IP2</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>kurbatov</t>
+          <t>charaburaev</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -9854,13 +9707,13 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>41.96</v>
+        <v>178.74</v>
       </c>
       <c r="G3" t="n">
-        <v>3500</v>
+        <v>13600</v>
       </c>
       <c r="H3" t="n">
-        <v>3500</v>
+        <v>13600</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -9869,110 +9722,12 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>14.05.2026 23:53</t>
+          <t>25.06.2026 14:19</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Похоже, в поле 'Курс' вписана сумма сделки (3500.00) вместо реального курса</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>188170</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>OB-TPPY013IP2</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>charaburaev</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>USDT</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>178.74</v>
-      </c>
-      <c r="G4" t="n">
-        <v>13600</v>
-      </c>
-      <c r="H4" t="n">
-        <v>13600</v>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Telegram</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>25.06.2026 14:19</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
           <t>Похоже, в поле 'Курс' вписана сумма сделки (13600.00) вместо реального курса</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>221773</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>OS-3KWU45AWNW</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>akhmedov</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>USDT</t>
-        </is>
-      </c>
-      <c r="F5" t="n">
-        <v>10.7527</v>
-      </c>
-      <c r="G5" t="n">
-        <v>1000</v>
-      </c>
-      <c r="H5" t="n">
-        <v>1000</v>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>Telegram</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>19.07.2026 23:38</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Похоже, в поле 'Курс' вписана сумма сделки (1000.00) вместо реального курса</t>
         </is>
       </c>
     </row>
@@ -9987,7 +9742,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K15"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10160,16 +9915,16 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>122984</v>
+        <v>133680</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>OB-HWNNXLBWH</t>
+          <t>OB-BVGPBDGPEY</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>khabibullin</t>
+          <t>shaidullov</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -10183,13 +9938,13 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>196.8773</v>
+        <v>644.2021999999999</v>
       </c>
       <c r="G4" t="n">
-        <v>75.51000000000001</v>
+        <v>74.31999999999999</v>
       </c>
       <c r="H4" t="n">
-        <v>196.88</v>
+        <v>644.2</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -10198,27 +9953,27 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>07.05.2026 12:34</t>
+          <t>14.05.2026 10:02</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Похоже, в поле 'Сумма' вписано количество крипты (196.8773) вместо рублей</t>
+          <t>Похоже, в поле 'Сумма' вписано количество крипты (644.2022) вместо рублей</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>132122</v>
+        <v>151414</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>OB-WF5KKTRKO</t>
+          <t>OB-5HXR4XIZ53</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>khabibullin</t>
+          <t>shaidullov</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -10232,13 +9987,13 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>377.5752</v>
+        <v>1228.0052</v>
       </c>
       <c r="G5" t="n">
-        <v>75</v>
+        <v>74.25</v>
       </c>
       <c r="H5" t="n">
-        <v>377.58</v>
+        <v>1228</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -10247,32 +10002,32 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>13.05.2026 16:20</t>
+          <t>28.05.2026 20:35</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Похоже, в поле 'Сумма' вписано количество крипты (377.5752) вместо рублей</t>
+          <t>Похоже, в поле 'Сумма' вписано количество крипты (1228.0052) вместо рублей</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>133680</v>
+        <v>155200</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>OB-BVGPBDGPEY</t>
+          <t>OS-F4QNQMT74J</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>shaidullov</t>
+          <t>dron</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -10281,13 +10036,13 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>644.2021999999999</v>
+        <v>200</v>
       </c>
       <c r="G6" t="n">
-        <v>74.31999999999999</v>
+        <v>81.39</v>
       </c>
       <c r="H6" t="n">
-        <v>644.2</v>
+        <v>200</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -10296,32 +10051,32 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>14.05.2026 10:02</t>
+          <t>29.05.2026 22:31</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Похоже, в поле 'Сумма' вписано количество крипты (644.2022) вместо рублей</t>
+          <t>Похоже, в поле 'Сумма' вписано количество крипты (200.0000) вместо рублей</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>137075</v>
+        <v>166004</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>OB-3L70JT07NU</t>
+          <t>OS-2A2TRB4H95</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>khabibullin</t>
+          <t>dron</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -10330,13 +10085,13 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>195.5192</v>
+        <v>1205.2549</v>
       </c>
       <c r="G7" t="n">
-        <v>73.5</v>
+        <v>82.97</v>
       </c>
       <c r="H7" t="n">
-        <v>195.52</v>
+        <v>1205.25</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -10345,47 +10100,47 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>17.05.2026 09:00</t>
+          <t>10.06.2026 01:04</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Похоже, в поле 'Сумма' вписано количество крипты (195.5192) вместо рублей</t>
+          <t>Похоже, в поле 'Сумма' вписано количество крипты (1205.2549) вместо рублей</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>151414</v>
+        <v>166049</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>OB-5HXR4XIZ53</t>
+          <t>OS-LTLOZ3GFY5</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>shaidullov</t>
+          <t>dron</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>SELL</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>USDT</t>
+          <t>TON</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>1228.0052</v>
+        <v>70</v>
       </c>
       <c r="G8" t="n">
-        <v>74.25</v>
+        <v>140.66</v>
       </c>
       <c r="H8" t="n">
-        <v>1228</v>
+        <v>70</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
@@ -10394,27 +10149,27 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>28.05.2026 20:35</t>
+          <t>10.06.2026 14:21</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Похоже, в поле 'Сумма' вписано количество крипты (1228.0052) вместо рублей</t>
+          <t>Похоже, в поле 'Сумма' вписано количество крипты (70.0000) вместо рублей</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>155200</v>
+        <v>193197</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>OS-F4QNQMT74J</t>
+          <t>OS-KBB4R5FGWD</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>dron</t>
+          <t>salatgereev_isa</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -10428,13 +10183,13 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>200</v>
+        <v>275.5453</v>
       </c>
       <c r="G9" t="n">
-        <v>81.39</v>
+        <v>87.09999999999999</v>
       </c>
       <c r="H9" t="n">
-        <v>200</v>
+        <v>275.55</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -10443,27 +10198,27 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>29.05.2026 22:31</t>
+          <t>25.06.2026 09:46</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Похоже, в поле 'Сумма' вписано количество крипты (200.0000) вместо рублей</t>
+          <t>Похоже, в поле 'Сумма' вписано количество крипты (275.5453) вместо рублей</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>166004</v>
+        <v>204756</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>OS-2A2TRB4H95</t>
+          <t>OS-0WD3E0YJ2U</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>dron</t>
+          <t>salatgereev_isa</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -10477,13 +10232,13 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>1205.2549</v>
+        <v>173.8123</v>
       </c>
       <c r="G10" t="n">
-        <v>82.97</v>
+        <v>86.3</v>
       </c>
       <c r="H10" t="n">
-        <v>1205.25</v>
+        <v>173.81</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -10492,27 +10247,27 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>10.06.2026 01:04</t>
+          <t>08.07.2026 07:58</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Похоже, в поле 'Сумма' вписано количество крипты (1205.2549) вместо рублей</t>
+          <t>Похоже, в поле 'Сумма' вписано количество крипты (173.8123) вместо рублей</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>166049</v>
+        <v>226350</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>OS-LTLOZ3GFY5</t>
+          <t>OS-RAPSVQWRKI</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>dron</t>
+          <t>charaburaev</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -10522,17 +10277,17 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>TON</t>
+          <t>USDT</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>70</v>
+        <v>25</v>
       </c>
       <c r="G11" t="n">
-        <v>140.66</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="H11" t="n">
-        <v>70</v>
+        <v>25</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -10541,206 +10296,10 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>10.06.2026 14:21</t>
+          <t>22.07.2026 14:01</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
-        <is>
-          <t>Похоже, в поле 'Сумма' вписано количество крипты (70.0000) вместо рублей</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="n">
-        <v>193197</v>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>OS-KBB4R5FGWD</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>salatgereev_isa</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>USDT</t>
-        </is>
-      </c>
-      <c r="F12" t="n">
-        <v>275.5453</v>
-      </c>
-      <c r="G12" t="n">
-        <v>87.09999999999999</v>
-      </c>
-      <c r="H12" t="n">
-        <v>275.55</v>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>Telegram</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>25.06.2026 09:46</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>Похоже, в поле 'Сумма' вписано количество крипты (275.5453) вместо рублей</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="n">
-        <v>193471</v>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>OB-5TBDPWA8NQ</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>ohannisyan</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>USDT</t>
-        </is>
-      </c>
-      <c r="F13" t="n">
-        <v>322.0721</v>
-      </c>
-      <c r="G13" t="n">
-        <v>76.93000000000001</v>
-      </c>
-      <c r="H13" t="n">
-        <v>322.07</v>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>Telegram</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>30.06.2026 22:14</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>Похоже, в поле 'Сумма' вписано количество крипты (322.0721) вместо рублей</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="n">
-        <v>204756</v>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>OS-0WD3E0YJ2U</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>salatgereev_isa</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>USDT</t>
-        </is>
-      </c>
-      <c r="F14" t="n">
-        <v>173.8123</v>
-      </c>
-      <c r="G14" t="n">
-        <v>86.3</v>
-      </c>
-      <c r="H14" t="n">
-        <v>173.81</v>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>Telegram</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>08.07.2026 07:58</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>Похоже, в поле 'Сумма' вписано количество крипты (173.8123) вместо рублей</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="n">
-        <v>226350</v>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>OS-RAPSVQWRKI</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>charaburaev</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>USDT</t>
-        </is>
-      </c>
-      <c r="F15" t="n">
-        <v>25</v>
-      </c>
-      <c r="G15" t="n">
-        <v>89.59999999999999</v>
-      </c>
-      <c r="H15" t="n">
-        <v>25</v>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>Telegram</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>22.07.2026 14:01</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr">
         <is>
           <t>Похоже, в поле 'Сумма' вписано количество крипты (25.0000) вместо рублей</t>
         </is>
@@ -10757,7 +10316,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11077,16 +10636,16 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>142338</v>
+        <v>196390</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>OS-LTUNEOQUWO</t>
+          <t>OS-GHB1B1PHDQ</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>arslangereev</t>
+          <t>nasibov</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -11100,13 +10659,13 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>1000</v>
+        <v>56.81</v>
       </c>
       <c r="G7" t="n">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="H7" t="n">
-        <v>8200</v>
+        <v>50000</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -11115,108 +10674,10 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>22.05.2026 07:34</t>
+          <t>03.07.2026 10:08</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
-        <is>
-          <t>Сумма отличается от ожидаемой ровно в 0.1x - похоже на 'забытый ноль' при вводе</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>192273</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>OB-GHT30FAHX1</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>khabibullin</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>USDT</t>
-        </is>
-      </c>
-      <c r="F8" t="n">
-        <v>128.8998</v>
-      </c>
-      <c r="G8" t="n">
-        <v>7815</v>
-      </c>
-      <c r="H8" t="n">
-        <v>10164.18</v>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>Telegram</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>29.06.2026 14:10</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>Сумма отличается от ожидаемой ровно в 0.01x - похоже на 'забытый ноль' при вводе</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>196390</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>OS-GHB1B1PHDQ</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>nasibov</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>USDT</t>
-        </is>
-      </c>
-      <c r="F9" t="n">
-        <v>56.81</v>
-      </c>
-      <c r="G9" t="n">
-        <v>88</v>
-      </c>
-      <c r="H9" t="n">
-        <v>50000</v>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>Telegram</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>03.07.2026 10:08</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
         <is>
           <t>Сумма отличается от ожидаемой ровно в 10x - похоже на 'забытый ноль' при вводе</t>
         </is>

</xml_diff>